<commit_message>
Add THAICON multi/PAC products (31 new rows, fix BTU/price/cassette bugs)
- Removed 36 wrong rows (Multi BTU=7 due to col mapping bug)
- Added outdoor (6), wall multi (2), cassette (3), duct (3),
  Balance On/off big (2), PAC cassette/duct/floor-ceiling (15) — total 31
- Fixed Multi sheet: col_kw=1→2, col_rrp=7→9
- Fixed dedup check to compare full 'THAICON TL-...' model name
- Fixed cassette Cyrillic МС detection via regex
- Total catalog: 522 products, THAICON: 60

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/splithub_master_template_MDV_filled_v2.xlsx
+++ b/splithub_master_template_MDV_filled_v2.xlsx
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA4913"/>
+  <dimension ref="A1:AA4877"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.5546875" customWidth="1" style="12" min="1" max="1"/>
@@ -57038,97 +57038,3570 @@
       </c>
     </row>
     <row r="493">
-      <c r="X493" s="1" t="n"/>
+      <c r="A493" t="n">
+        <v>1</v>
+      </c>
+      <c r="B493" t="n">
+        <v>1492</v>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>thaicon-rwb80</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>Balance On/off</t>
+        </is>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>THAICON TL-RWB80-NA</t>
+        </is>
+      </c>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>onoff</t>
+        </is>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K493" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L493" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="M493" t="n">
+        <v>27</v>
+      </c>
+      <c r="N493" t="inlineStr">
+        <is>
+          <t>8.21</t>
+        </is>
+      </c>
+      <c r="O493" t="n">
+        <v>70</v>
+      </c>
+      <c r="P493" t="n">
+        <v>80200</v>
+      </c>
+      <c r="Q493" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R493" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S493" t="inlineStr">
+        <is>
+          <t>Balance On/off On/Off 27 BTU · до 70 м²</t>
+        </is>
+      </c>
+      <c r="T493" t="inlineStr">
+        <is>
+          <t>EER/COP - класс А · обогрев до -7 °С · Wi-Fi ready · 5 скоростей · 3 года</t>
+        </is>
+      </c>
+      <c r="U493" t="inlineStr">
+        <is>
+          <t>Wi-Fi ready|5 скоростей вентилятора|R32 (20-70)/R410А(80-100)|EER/COP - класс А|обогрев до -7 °С|охлаждение от +15 °С|фильтр с ионами серебра|Гарантия - 3  года</t>
+        </is>
+      </c>
+      <c r="V493" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W493" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X493" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-balance.webp</t>
+        </is>
+      </c>
+      <c r="Y493" t="n">
+        <v>316</v>
+      </c>
     </row>
     <row r="494">
-      <c r="X494" s="1" t="n"/>
+      <c r="A494" t="n">
+        <v>1</v>
+      </c>
+      <c r="B494" t="n">
+        <v>1493</v>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>thaicon-rwb100</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>Balance On/off</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>THAICON TL-RWB100-NA</t>
+        </is>
+      </c>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>onoff</t>
+        </is>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K494" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L494" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="M494" t="n">
+        <v>36</v>
+      </c>
+      <c r="N494" t="inlineStr">
+        <is>
+          <t>10.55</t>
+        </is>
+      </c>
+      <c r="O494" t="n">
+        <v>100</v>
+      </c>
+      <c r="P494" t="n">
+        <v>99800</v>
+      </c>
+      <c r="Q494" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R494" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S494" t="inlineStr">
+        <is>
+          <t>Balance On/off On/Off 36 BTU · до 100 м²</t>
+        </is>
+      </c>
+      <c r="T494" t="inlineStr">
+        <is>
+          <t>EER/COP - класс А · обогрев до -7 °С · Wi-Fi ready · 5 скоростей · 3 года</t>
+        </is>
+      </c>
+      <c r="U494" t="inlineStr">
+        <is>
+          <t>Wi-Fi ready|5 скоростей вентилятора|R32 (20-70)/R410А(80-100)|EER/COP - класс А|обогрев до -7 °С|охлаждение от +15 °С|фильтр с ионами серебра|Гарантия - 3  года</t>
+        </is>
+      </c>
+      <c r="V494" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W494" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X494" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-balance.webp</t>
+        </is>
+      </c>
+      <c r="Y494" t="n">
+        <v>317</v>
+      </c>
     </row>
     <row r="495">
-      <c r="X495" s="1" t="n"/>
+      <c r="A495" t="n">
+        <v>1</v>
+      </c>
+      <c r="B495" t="n">
+        <v>1494</v>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>thaicon-mo2u40</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT outdoor</t>
+        </is>
+      </c>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>THAICON TL-MO2U40-FR</t>
+        </is>
+      </c>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>multi</t>
+        </is>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K495" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L495" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M495" t="n">
+        <v>14</v>
+      </c>
+      <c r="N495" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="O495" t="n">
+        <v>40</v>
+      </c>
+      <c r="P495" t="n">
+        <v>54900</v>
+      </c>
+      <c r="Q495" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R495" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S495" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT outdoor 14 BTU</t>
+        </is>
+      </c>
+      <c r="T495" t="inlineStr">
+        <is>
+          <t>THAICON · Мульти · Наружный блок · А++ · обогрев -20°С · R32</t>
+        </is>
+      </c>
+      <c r="U495" t="inlineStr">
+        <is>
+          <t>А++ класс энергоэффективности|Подключение до 5 внутренних блоков|Компрессоры GMCC/SANYO|Обогрев до -20°С|Охлаждение до -15°С|Защитная крышка вентилей|R32|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V495" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W495" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X495" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-multi.webp</t>
+        </is>
+      </c>
+      <c r="Y495" t="n">
+        <v>318</v>
+      </c>
     </row>
     <row r="496">
-      <c r="X496" s="1" t="n"/>
+      <c r="A496" t="n">
+        <v>1</v>
+      </c>
+      <c r="B496" t="n">
+        <v>1495</v>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>thaicon-mo2u50</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT outdoor</t>
+        </is>
+      </c>
+      <c r="G496" t="inlineStr">
+        <is>
+          <t>THAICON TL-MO2U50-FR</t>
+        </is>
+      </c>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>multi</t>
+        </is>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K496" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L496" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M496" t="n">
+        <v>18</v>
+      </c>
+      <c r="N496" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="O496" t="n">
+        <v>50</v>
+      </c>
+      <c r="P496" t="n">
+        <v>64400</v>
+      </c>
+      <c r="Q496" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R496" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S496" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT outdoor 18 BTU</t>
+        </is>
+      </c>
+      <c r="T496" t="inlineStr">
+        <is>
+          <t>THAICON · Мульти · Наружный блок · А++ · обогрев -20°С · R32</t>
+        </is>
+      </c>
+      <c r="U496" t="inlineStr">
+        <is>
+          <t>А++ класс энергоэффективности|Подключение до 5 внутренних блоков|Компрессоры GMCC/SANYO|Обогрев до -20°С|Охлаждение до -15°С|Защитная крышка вентилей|R32|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V496" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W496" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X496" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-multi.webp</t>
+        </is>
+      </c>
+      <c r="Y496" t="n">
+        <v>319</v>
+      </c>
     </row>
     <row r="497">
-      <c r="X497" s="1" t="n"/>
+      <c r="A497" t="n">
+        <v>1</v>
+      </c>
+      <c r="B497" t="n">
+        <v>1496</v>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>thaicon-mo3u70</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT outdoor</t>
+        </is>
+      </c>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>THAICON TL-MO3U70-FR</t>
+        </is>
+      </c>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>multi</t>
+        </is>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K497" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L497" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M497" t="n">
+        <v>21</v>
+      </c>
+      <c r="N497" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="O497" t="n">
+        <v>60</v>
+      </c>
+      <c r="P497" t="n">
+        <v>81000</v>
+      </c>
+      <c r="Q497" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R497" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S497" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT outdoor 21 BTU</t>
+        </is>
+      </c>
+      <c r="T497" t="inlineStr">
+        <is>
+          <t>THAICON · Мульти · Наружный блок · А++ · обогрев -20°С · R32</t>
+        </is>
+      </c>
+      <c r="U497" t="inlineStr">
+        <is>
+          <t>А++ класс энергоэффективности|Подключение до 5 внутренних блоков|Компрессоры GMCC/SANYO|Обогрев до -20°С|Охлаждение до -15°С|Защитная крышка вентилей|R32|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V497" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W497" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X497" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-multi.webp</t>
+        </is>
+      </c>
+      <c r="Y497" t="n">
+        <v>320</v>
+      </c>
     </row>
     <row r="498">
-      <c r="X498" s="1" t="n"/>
+      <c r="A498" t="n">
+        <v>1</v>
+      </c>
+      <c r="B498" t="n">
+        <v>1497</v>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>thaicon-mo3u80</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT outdoor</t>
+        </is>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>THAICON TL-MO3U80-FR</t>
+        </is>
+      </c>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>multi</t>
+        </is>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K498" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L498" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M498" t="n">
+        <v>27</v>
+      </c>
+      <c r="N498" t="inlineStr">
+        <is>
+          <t>7.9</t>
+        </is>
+      </c>
+      <c r="O498" t="n">
+        <v>70</v>
+      </c>
+      <c r="P498" t="n">
+        <v>94200</v>
+      </c>
+      <c r="Q498" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R498" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S498" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT outdoor 27 BTU</t>
+        </is>
+      </c>
+      <c r="T498" t="inlineStr">
+        <is>
+          <t>THAICON · Мульти · Наружный блок · А++ · обогрев -20°С · R32</t>
+        </is>
+      </c>
+      <c r="U498" t="inlineStr">
+        <is>
+          <t>А++ класс энергоэффективности|Подключение до 5 внутренних блоков|Компрессоры GMCC/SANYO|Обогрев до -20°С|Охлаждение до -15°С|Защитная крышка вентилей|R32|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V498" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W498" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X498" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-multi.webp</t>
+        </is>
+      </c>
+      <c r="Y498" t="n">
+        <v>321</v>
+      </c>
     </row>
     <row r="499">
-      <c r="X499" s="1" t="n"/>
+      <c r="A499" t="n">
+        <v>1</v>
+      </c>
+      <c r="B499" t="n">
+        <v>1498</v>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>thaicon-mo4u100</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT outdoor</t>
+        </is>
+      </c>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>THAICON TL-MO4U100-FR</t>
+        </is>
+      </c>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>multi</t>
+        </is>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K499" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L499" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M499" t="n">
+        <v>32</v>
+      </c>
+      <c r="N499" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="O499" t="n">
+        <v>90</v>
+      </c>
+      <c r="P499" t="n">
+        <v>130200</v>
+      </c>
+      <c r="Q499" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R499" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S499" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT outdoor 32 BTU</t>
+        </is>
+      </c>
+      <c r="T499" t="inlineStr">
+        <is>
+          <t>THAICON · Мульти · Наружный блок · А++ · обогрев -20°С · R32</t>
+        </is>
+      </c>
+      <c r="U499" t="inlineStr">
+        <is>
+          <t>А++ класс энергоэффективности|Подключение до 5 внутренних блоков|Компрессоры GMCC/SANYO|Обогрев до -20°С|Охлаждение до -15°С|Защитная крышка вентилей|R32|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V499" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W499" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X499" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-multi.webp</t>
+        </is>
+      </c>
+      <c r="Y499" t="n">
+        <v>322</v>
+      </c>
     </row>
     <row r="500">
-      <c r="X500" s="1" t="n"/>
+      <c r="A500" t="n">
+        <v>1</v>
+      </c>
+      <c r="B500" t="n">
+        <v>1499</v>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>thaicon-mo5u120</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT outdoor</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>THAICON TL-MO5U120-FR</t>
+        </is>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>multi</t>
+        </is>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K500" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L500" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M500" t="n">
+        <v>42</v>
+      </c>
+      <c r="N500" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="O500" t="n">
+        <v>120</v>
+      </c>
+      <c r="P500" t="n">
+        <v>163300</v>
+      </c>
+      <c r="Q500" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R500" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S500" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT outdoor 42 BTU</t>
+        </is>
+      </c>
+      <c r="T500" t="inlineStr">
+        <is>
+          <t>THAICON · Мульти · Наружный блок · А++ · обогрев -20°С · R32</t>
+        </is>
+      </c>
+      <c r="U500" t="inlineStr">
+        <is>
+          <t>А++ класс энергоэффективности|Подключение до 5 внутренних блоков|Компрессоры GMCC/SANYO|Обогрев до -20°С|Охлаждение до -15°С|Защитная крышка вентилей|R32|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V500" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W500" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X500" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-multi.webp</t>
+        </is>
+      </c>
+      <c r="Y500" t="n">
+        <v>323</v>
+      </c>
     </row>
     <row r="501">
-      <c r="X501" s="1" t="n"/>
+      <c r="A501" t="n">
+        <v>1</v>
+      </c>
+      <c r="B501" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>thaicon-rwp20</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>PHANTOM inverter</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>THAICON TL-RWP20-FR</t>
+        </is>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>multi</t>
+        </is>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K501" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L501" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M501" t="n">
+        <v>7</v>
+      </c>
+      <c r="N501" t="inlineStr">
+        <is>
+          <t>2.05</t>
+        </is>
+      </c>
+      <c r="O501" t="n">
+        <v>20</v>
+      </c>
+      <c r="P501" t="n">
+        <v>19000</v>
+      </c>
+      <c r="Q501" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R501" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S501" t="inlineStr">
+        <is>
+          <t>PHANTOM inverter Инвертор 7 BTU · до 20 м²</t>
+        </is>
+      </c>
+      <c r="T501" t="inlineStr">
+        <is>
+          <t>Черный глянец · Full DC Inverter ·  SEER А++/SCOP A+ · обогрев до -20 °С · 7 скоростей · 4D Air Flow · Wi-Fi-модуль · ионизатор Dual Stream · 4 года</t>
+        </is>
+      </c>
+      <c r="U501" t="inlineStr">
+        <is>
+          <t>Cтильный дизайн с глянцевой панелью|Full DC Inverter / R32|SEER А++/SCOP A+|обогрев до -20 °С|охлаждение до -15 °С  
+7 скоростей вентилятора|4D Air Flow|встроенный Wi-Fi-модуль|тихие в работе от 22 дБ(А)|биполярный ионизатор Dual Stream|фильтр с ионами серебра|угольный фильтр|самоочистка 56 °С|Гарантия - 4 года</t>
+        </is>
+      </c>
+      <c r="V501" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W501" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X501" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-phantom.webp</t>
+        </is>
+      </c>
+      <c r="Y501" t="n">
+        <v>324</v>
+      </c>
     </row>
     <row r="502">
-      <c r="X502" s="1" t="n"/>
+      <c r="A502" t="n">
+        <v>1</v>
+      </c>
+      <c r="B502" t="n">
+        <v>1501</v>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>thaicon-rwc20</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>Comfort Plus Invertor</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>THAICON TL-RWC20-FR</t>
+        </is>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>multi</t>
+        </is>
+      </c>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J502" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K502" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L502" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M502" t="n">
+        <v>7</v>
+      </c>
+      <c r="N502" t="inlineStr">
+        <is>
+          <t>2.05</t>
+        </is>
+      </c>
+      <c r="O502" t="n">
+        <v>20</v>
+      </c>
+      <c r="P502" t="n">
+        <v>18200</v>
+      </c>
+      <c r="Q502" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R502" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S502" t="inlineStr">
+        <is>
+          <t>Comfort Plus Invertor Инвертор 7 BTU · до 20 м²</t>
+        </is>
+      </c>
+      <c r="T502" t="inlineStr">
+        <is>
+          <t>AI Eco Mind(ИИ) · Wi-fi встроенный · Автоочистка · 4D Air Flow · Full DC Inverter · R32 · SEER А++/SCOP A+  · обогрев до -20 °С</t>
+        </is>
+      </c>
+      <c r="U502" t="inlineStr">
+        <is>
+          <t>Full DC Inverter / R32|SEER А++/SCOP A+|обогрев до -20 °С|охлаждение до -15 °С|7 скоростей вентилятора|4D Air Flow|встроенный Wi-Fi-модуль|тихие в работе от 22 дБ(А)|биполярный ионизатор Dual Stream|самоочистка 56 °С|AI EcoMind|Гарантия 4 ГОДА</t>
+        </is>
+      </c>
+      <c r="V502" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W502" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X502" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-comfort-plus.webp</t>
+        </is>
+      </c>
+      <c r="Y502" t="n">
+        <v>325</v>
+      </c>
     </row>
     <row r="503">
-      <c r="X503" s="1" t="n"/>
+      <c r="A503" t="n">
+        <v>1</v>
+      </c>
+      <c r="B503" t="n">
+        <v>1502</v>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>thaicon-mс25</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT cassette</t>
+        </is>
+      </c>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>THAICON TL-MС25-FR</t>
+        </is>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>multi</t>
+        </is>
+      </c>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J503" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K503" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L503" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M503" t="n">
+        <v>9</v>
+      </c>
+      <c r="N503" t="inlineStr">
+        <is>
+          <t>2.64</t>
+        </is>
+      </c>
+      <c r="O503" t="n">
+        <v>25</v>
+      </c>
+      <c r="P503" t="n">
+        <v>45000</v>
+      </c>
+      <c r="Q503" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R503" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S503" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT cassette Инвертор 9 BTU · до 25 м²</t>
+        </is>
+      </c>
+      <c r="T503" t="inlineStr">
+        <is>
+          <t>THAICON · Мульти · Кассетный · 4-поток · встроенная помпа · R32</t>
+        </is>
+      </c>
+      <c r="U503" t="inlineStr">
+        <is>
+          <t>Кассетный внутренний блок мультисплит|360° распределение воздуха|Встроенная дренажная помпа|Противопылевой фильтр|Декоративная панель в комплекте|R32|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V503" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W503" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X503" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-multi-cassette.webp</t>
+        </is>
+      </c>
+      <c r="Y503" t="n">
+        <v>326</v>
+      </c>
     </row>
     <row r="504">
-      <c r="X504" s="1" t="n"/>
+      <c r="A504" t="n">
+        <v>1</v>
+      </c>
+      <c r="B504" t="n">
+        <v>1503</v>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>thaicon-mс35</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT cassette</t>
+        </is>
+      </c>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>THAICON TL-MС35-FR</t>
+        </is>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>multi</t>
+        </is>
+      </c>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J504" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K504" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L504" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M504" t="n">
+        <v>12</v>
+      </c>
+      <c r="N504" t="inlineStr">
+        <is>
+          <t>3.52</t>
+        </is>
+      </c>
+      <c r="O504" t="n">
+        <v>35</v>
+      </c>
+      <c r="P504" t="n">
+        <v>49600</v>
+      </c>
+      <c r="Q504" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R504" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S504" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT cassette Инвертор 12 BTU · до 35 м²</t>
+        </is>
+      </c>
+      <c r="T504" t="inlineStr">
+        <is>
+          <t>THAICON · Мульти · Кассетный · 4-поток · встроенная помпа · R32</t>
+        </is>
+      </c>
+      <c r="U504" t="inlineStr">
+        <is>
+          <t>Кассетный внутренний блок мультисплит|360° распределение воздуха|Встроенная дренажная помпа|Противопылевой фильтр|Декоративная панель в комплекте|R32|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V504" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W504" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X504" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-multi-cassette.webp</t>
+        </is>
+      </c>
+      <c r="Y504" t="n">
+        <v>327</v>
+      </c>
     </row>
     <row r="505">
-      <c r="X505" s="1" t="n"/>
+      <c r="A505" t="n">
+        <v>1</v>
+      </c>
+      <c r="B505" t="n">
+        <v>1504</v>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>thaicon-mс50</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT cassette</t>
+        </is>
+      </c>
+      <c r="G505" t="inlineStr">
+        <is>
+          <t>THAICON TL-MС50-FR</t>
+        </is>
+      </c>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>multi</t>
+        </is>
+      </c>
+      <c r="I505" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J505" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K505" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L505" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M505" t="n">
+        <v>18</v>
+      </c>
+      <c r="N505" t="inlineStr">
+        <is>
+          <t>5.27</t>
+        </is>
+      </c>
+      <c r="O505" t="n">
+        <v>50</v>
+      </c>
+      <c r="P505" t="n">
+        <v>54200</v>
+      </c>
+      <c r="Q505" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R505" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S505" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT cassette Инвертор 18 BTU · до 50 м²</t>
+        </is>
+      </c>
+      <c r="T505" t="inlineStr">
+        <is>
+          <t>THAICON · Мульти · Кассетный · 4-поток · встроенная помпа · R32</t>
+        </is>
+      </c>
+      <c r="U505" t="inlineStr">
+        <is>
+          <t>Кассетный внутренний блок мультисплит|360° распределение воздуха|Встроенная дренажная помпа|Противопылевой фильтр|Декоративная панель в комплекте|R32|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V505" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W505" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X505" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-multi-cassette.webp</t>
+        </is>
+      </c>
+      <c r="Y505" t="n">
+        <v>328</v>
+      </c>
     </row>
     <row r="506">
-      <c r="X506" s="1" t="n"/>
+      <c r="A506" t="n">
+        <v>1</v>
+      </c>
+      <c r="B506" t="n">
+        <v>1505</v>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>thaicon-md25</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT duct</t>
+        </is>
+      </c>
+      <c r="G506" t="inlineStr">
+        <is>
+          <t>THAICON TL-MD25-FR</t>
+        </is>
+      </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>multi</t>
+        </is>
+      </c>
+      <c r="I506" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J506" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K506" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L506" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M506" t="n">
+        <v>9</v>
+      </c>
+      <c r="N506" t="inlineStr">
+        <is>
+          <t>2.64</t>
+        </is>
+      </c>
+      <c r="O506" t="n">
+        <v>25</v>
+      </c>
+      <c r="P506" t="n">
+        <v>37000</v>
+      </c>
+      <c r="Q506" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R506" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S506" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT duct Инвертор 9 BTU · до 25 м²</t>
+        </is>
+      </c>
+      <c r="T506" t="inlineStr">
+        <is>
+          <t>THAICON · Мульти · Канальный · Скрытый монтаж · R32</t>
+        </is>
+      </c>
+      <c r="U506" t="inlineStr">
+        <is>
+          <t>Канальный внутренний блок мультисплит|Скрытый монтаж|Встроенная дренажная помпа|Противопылевой фильтр|Приёмник ИК-сигнала в комплекте|R32|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V506" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W506" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X506" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-multi-duct.webp</t>
+        </is>
+      </c>
+      <c r="Y506" t="n">
+        <v>329</v>
+      </c>
     </row>
     <row r="507">
-      <c r="X507" s="1" t="n"/>
+      <c r="A507" t="n">
+        <v>1</v>
+      </c>
+      <c r="B507" t="n">
+        <v>1506</v>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>thaicon-md35</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT duct</t>
+        </is>
+      </c>
+      <c r="G507" t="inlineStr">
+        <is>
+          <t>THAICON TL-MD35-FR</t>
+        </is>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>multi</t>
+        </is>
+      </c>
+      <c r="I507" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J507" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K507" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L507" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M507" t="n">
+        <v>12</v>
+      </c>
+      <c r="N507" t="inlineStr">
+        <is>
+          <t>3.52</t>
+        </is>
+      </c>
+      <c r="O507" t="n">
+        <v>35</v>
+      </c>
+      <c r="P507" t="n">
+        <v>38400</v>
+      </c>
+      <c r="Q507" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R507" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S507" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT duct Инвертор 12 BTU · до 35 м²</t>
+        </is>
+      </c>
+      <c r="T507" t="inlineStr">
+        <is>
+          <t>THAICON · Мульти · Канальный · Скрытый монтаж · R32</t>
+        </is>
+      </c>
+      <c r="U507" t="inlineStr">
+        <is>
+          <t>Канальный внутренний блок мультисплит|Скрытый монтаж|Встроенная дренажная помпа|Противопылевой фильтр|Приёмник ИК-сигнала в комплекте|R32|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V507" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W507" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X507" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-multi-duct.webp</t>
+        </is>
+      </c>
+      <c r="Y507" t="n">
+        <v>330</v>
+      </c>
     </row>
     <row r="508">
-      <c r="X508" s="1" t="n"/>
+      <c r="A508" t="n">
+        <v>1</v>
+      </c>
+      <c r="B508" t="n">
+        <v>1507</v>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>thaicon-md50</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT duct</t>
+        </is>
+      </c>
+      <c r="G508" t="inlineStr">
+        <is>
+          <t>THAICON TL-MD50-FR</t>
+        </is>
+      </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>multi</t>
+        </is>
+      </c>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J508" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K508" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L508" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M508" t="n">
+        <v>18</v>
+      </c>
+      <c r="N508" t="inlineStr">
+        <is>
+          <t>5.27</t>
+        </is>
+      </c>
+      <c r="O508" t="n">
+        <v>50</v>
+      </c>
+      <c r="P508" t="n">
+        <v>42200</v>
+      </c>
+      <c r="Q508" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R508" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S508" t="inlineStr">
+        <is>
+          <t>MULTI COMFORT duct Инвертор 18 BTU · до 50 м²</t>
+        </is>
+      </c>
+      <c r="T508" t="inlineStr">
+        <is>
+          <t>THAICON · Мульти · Канальный · Скрытый монтаж · R32</t>
+        </is>
+      </c>
+      <c r="U508" t="inlineStr">
+        <is>
+          <t>Канальный внутренний блок мультисплит|Скрытый монтаж|Встроенная дренажная помпа|Противопылевой фильтр|Приёмник ИК-сигнала в комплекте|R32|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V508" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W508" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X508" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-multi-duct.webp</t>
+        </is>
+      </c>
+      <c r="Y508" t="n">
+        <v>331</v>
+      </c>
     </row>
     <row r="509">
-      <c r="X509" s="1" t="n"/>
+      <c r="A509" t="n">
+        <v>1</v>
+      </c>
+      <c r="B509" t="n">
+        <v>1508</v>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>thaicon-pc50</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>SYNERGY cassette</t>
+        </is>
+      </c>
+      <c r="G509" t="inlineStr">
+        <is>
+          <t>THAICON TL-PC50-FR</t>
+        </is>
+      </c>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>pac_inv</t>
+        </is>
+      </c>
+      <c r="I509" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J509" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K509" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L509" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M509" t="n">
+        <v>18</v>
+      </c>
+      <c r="N509" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="O509" t="n">
+        <v>50</v>
+      </c>
+      <c r="P509" t="n">
+        <v>76500</v>
+      </c>
+      <c r="Q509" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R509" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S509" t="inlineStr">
+        <is>
+          <t>SYNERGY cassette Инвертор 18 BTU · до 50 м²</t>
+        </is>
+      </c>
+      <c r="T509" t="inlineStr">
+        <is>
+          <t>DC Inverter · 360° поток · LED-дисплей · ИК-пульт · обогрев -15°С · R32 · 3 года</t>
+        </is>
+      </c>
+      <c r="U509" t="inlineStr">
+        <is>
+          <t>DC Inverter / R32|Кассетный тип 360°|Обогрев до -15°С|Охлаждение до -15°С|LED-дисплей|ИК-пульт и декоративная панель в комплекте|Встроенная дренажная помпа|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V509" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W509" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X509" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-synergy-cassette.webp</t>
+        </is>
+      </c>
+      <c r="Y509" t="n">
+        <v>332</v>
+      </c>
     </row>
     <row r="510">
-      <c r="X510" s="1" t="n"/>
+      <c r="A510" t="n">
+        <v>1</v>
+      </c>
+      <c r="B510" t="n">
+        <v>1509</v>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>thaicon-pc70</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>SYNERGY cassette</t>
+        </is>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>THAICON TL-PC70-FR</t>
+        </is>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>pac_inv</t>
+        </is>
+      </c>
+      <c r="I510" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J510" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K510" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L510" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M510" t="n">
+        <v>24</v>
+      </c>
+      <c r="N510" t="inlineStr">
+        <is>
+          <t>7.03</t>
+        </is>
+      </c>
+      <c r="O510" t="n">
+        <v>65</v>
+      </c>
+      <c r="P510" t="n">
+        <v>94600</v>
+      </c>
+      <c r="Q510" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R510" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S510" t="inlineStr">
+        <is>
+          <t>SYNERGY cassette Инвертор 24 BTU · до 65 м²</t>
+        </is>
+      </c>
+      <c r="T510" t="inlineStr">
+        <is>
+          <t>DC Inverter · 360° поток · LED-дисплей · ИК-пульт · обогрев -15°С · R32 · 3 года</t>
+        </is>
+      </c>
+      <c r="U510" t="inlineStr">
+        <is>
+          <t>DC Inverter / R32|Кассетный тип 360°|Обогрев до -15°С|Охлаждение до -15°С|LED-дисплей|ИК-пульт и декоративная панель в комплекте|Встроенная дренажная помпа|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V510" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W510" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X510" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-synergy-cassette.webp</t>
+        </is>
+      </c>
+      <c r="Y510" t="n">
+        <v>333</v>
+      </c>
     </row>
     <row r="511">
-      <c r="X511" s="1" t="n"/>
+      <c r="A511" t="n">
+        <v>1</v>
+      </c>
+      <c r="B511" t="n">
+        <v>1510</v>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>thaicon-pc100</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>SYNERGY cassette</t>
+        </is>
+      </c>
+      <c r="G511" t="inlineStr">
+        <is>
+          <t>THAICON TL-PC100-FR</t>
+        </is>
+      </c>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>pac_inv</t>
+        </is>
+      </c>
+      <c r="I511" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J511" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K511" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L511" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M511" t="n">
+        <v>36</v>
+      </c>
+      <c r="N511" t="inlineStr">
+        <is>
+          <t>10.55</t>
+        </is>
+      </c>
+      <c r="O511" t="n">
+        <v>100</v>
+      </c>
+      <c r="P511" t="n">
+        <v>131700</v>
+      </c>
+      <c r="Q511" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R511" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S511" t="inlineStr">
+        <is>
+          <t>SYNERGY cassette Инвертор 36 BTU · до 100 м²</t>
+        </is>
+      </c>
+      <c r="T511" t="inlineStr">
+        <is>
+          <t>DC Inverter · 360° поток · LED-дисплей · ИК-пульт · обогрев -15°С · R32 · 3 года</t>
+        </is>
+      </c>
+      <c r="U511" t="inlineStr">
+        <is>
+          <t>DC Inverter / R32|Кассетный тип 360°|Обогрев до -15°С|Охлаждение до -15°С|LED-дисплей|ИК-пульт и декоративная панель в комплекте|Встроенная дренажная помпа|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V511" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W511" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X511" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-synergy-cassette.webp</t>
+        </is>
+      </c>
+      <c r="Y511" t="n">
+        <v>334</v>
+      </c>
     </row>
     <row r="512">
-      <c r="X512" s="1" t="n"/>
+      <c r="A512" t="n">
+        <v>1</v>
+      </c>
+      <c r="B512" t="n">
+        <v>1511</v>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>thaicon-pc140</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>SYNERGY cassette</t>
+        </is>
+      </c>
+      <c r="G512" t="inlineStr">
+        <is>
+          <t>THAICON TL-PC140-FR4</t>
+        </is>
+      </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>pac_inv</t>
+        </is>
+      </c>
+      <c r="I512" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J512" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K512" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L512" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M512" t="n">
+        <v>48</v>
+      </c>
+      <c r="N512" t="inlineStr">
+        <is>
+          <t>14.07</t>
+        </is>
+      </c>
+      <c r="O512" t="n">
+        <v>130</v>
+      </c>
+      <c r="P512" t="n">
+        <v>166600</v>
+      </c>
+      <c r="Q512" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R512" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S512" t="inlineStr">
+        <is>
+          <t>SYNERGY cassette Инвертор 48 BTU · до 130 м²</t>
+        </is>
+      </c>
+      <c r="T512" t="inlineStr">
+        <is>
+          <t>DC Inverter · 360° поток · LED-дисплей · ИК-пульт · обогрев -15°С · R32 · 3 года</t>
+        </is>
+      </c>
+      <c r="U512" t="inlineStr">
+        <is>
+          <t>DC Inverter / R32|Кассетный тип 360°|Обогрев до -15°С|Охлаждение до -15°С|LED-дисплей|ИК-пульт и декоративная панель в комплекте|Встроенная дренажная помпа|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V512" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W512" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X512" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-synergy-cassette.webp</t>
+        </is>
+      </c>
+      <c r="Y512" t="n">
+        <v>335</v>
+      </c>
     </row>
     <row r="513">
-      <c r="X513" s="1" t="n"/>
+      <c r="A513" t="n">
+        <v>1</v>
+      </c>
+      <c r="B513" t="n">
+        <v>1512</v>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>thaicon-pc170</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>SYNERGY cassette</t>
+        </is>
+      </c>
+      <c r="G513" t="inlineStr">
+        <is>
+          <t>THAICON TL-PC170-FR4</t>
+        </is>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>pac_inv</t>
+        </is>
+      </c>
+      <c r="I513" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J513" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K513" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L513" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M513" t="n">
+        <v>60</v>
+      </c>
+      <c r="N513" t="inlineStr">
+        <is>
+          <t>16.12</t>
+        </is>
+      </c>
+      <c r="O513" t="n">
+        <v>160</v>
+      </c>
+      <c r="P513" t="n">
+        <v>182500</v>
+      </c>
+      <c r="Q513" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R513" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S513" t="inlineStr">
+        <is>
+          <t>SYNERGY cassette Инвертор 60 BTU · до 160 м²</t>
+        </is>
+      </c>
+      <c r="T513" t="inlineStr">
+        <is>
+          <t>DC Inverter · 360° поток · LED-дисплей · ИК-пульт · обогрев -15°С · R32 · 3 года</t>
+        </is>
+      </c>
+      <c r="U513" t="inlineStr">
+        <is>
+          <t>DC Inverter / R32|Кассетный тип 360°|Обогрев до -15°С|Охлаждение до -15°С|LED-дисплей|ИК-пульт и декоративная панель в комплекте|Встроенная дренажная помпа|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V513" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W513" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X513" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-synergy-cassette.webp</t>
+        </is>
+      </c>
+      <c r="Y513" t="n">
+        <v>336</v>
+      </c>
     </row>
     <row r="514">
-      <c r="X514" s="1" t="n"/>
+      <c r="A514" t="n">
+        <v>1</v>
+      </c>
+      <c r="B514" t="n">
+        <v>1513</v>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>thaicon-pd50</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>SYNERGY duct</t>
+        </is>
+      </c>
+      <c r="G514" t="inlineStr">
+        <is>
+          <t>THAICON TL-PD50-FR</t>
+        </is>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>pac_inv</t>
+        </is>
+      </c>
+      <c r="I514" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J514" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K514" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L514" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M514" t="n">
+        <v>18</v>
+      </c>
+      <c r="N514" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="O514" t="n">
+        <v>50</v>
+      </c>
+      <c r="P514" t="n">
+        <v>80500</v>
+      </c>
+      <c r="Q514" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R514" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S514" t="inlineStr">
+        <is>
+          <t>SYNERGY duct Инвертор 18 BTU · до 50 м²</t>
+        </is>
+      </c>
+      <c r="T514" t="inlineStr">
+        <is>
+          <t>DC Inverter · Канальный · до 200 Па · проводной пульт · обогрев -15°С · R32 · 3 года</t>
+        </is>
+      </c>
+      <c r="U514" t="inlineStr">
+        <is>
+          <t>DC Inverter / R32|Канальный тип|Обогрев до -15°С|Охлаждение до -15°С|Встроенная дренажная помпа|Статическое давление до 200 Па|Проводной пульт в комплекте|Приёмник ИК-сигнала|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V514" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W514" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X514" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-synergy-duct.webp</t>
+        </is>
+      </c>
+      <c r="Y514" t="n">
+        <v>337</v>
+      </c>
     </row>
     <row r="515">
-      <c r="X515" s="1" t="n"/>
+      <c r="A515" t="n">
+        <v>1</v>
+      </c>
+      <c r="B515" t="n">
+        <v>1514</v>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>thaicon-pd70</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>SYNERGY duct</t>
+        </is>
+      </c>
+      <c r="G515" t="inlineStr">
+        <is>
+          <t>THAICON TL-PD70-FR</t>
+        </is>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>pac_inv</t>
+        </is>
+      </c>
+      <c r="I515" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J515" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K515" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L515" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M515" t="n">
+        <v>24</v>
+      </c>
+      <c r="N515" t="inlineStr">
+        <is>
+          <t>7.03</t>
+        </is>
+      </c>
+      <c r="O515" t="n">
+        <v>65</v>
+      </c>
+      <c r="P515" t="n">
+        <v>101200</v>
+      </c>
+      <c r="Q515" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R515" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S515" t="inlineStr">
+        <is>
+          <t>SYNERGY duct Инвертор 24 BTU · до 65 м²</t>
+        </is>
+      </c>
+      <c r="T515" t="inlineStr">
+        <is>
+          <t>DC Inverter · Канальный · до 200 Па · проводной пульт · обогрев -15°С · R32 · 3 года</t>
+        </is>
+      </c>
+      <c r="U515" t="inlineStr">
+        <is>
+          <t>DC Inverter / R32|Канальный тип|Обогрев до -15°С|Охлаждение до -15°С|Встроенная дренажная помпа|Статическое давление до 200 Па|Проводной пульт в комплекте|Приёмник ИК-сигнала|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V515" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W515" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X515" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-synergy-duct.webp</t>
+        </is>
+      </c>
+      <c r="Y515" t="n">
+        <v>338</v>
+      </c>
     </row>
     <row r="516">
-      <c r="X516" s="1" t="n"/>
+      <c r="A516" t="n">
+        <v>1</v>
+      </c>
+      <c r="B516" t="n">
+        <v>1515</v>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>thaicon-pd100</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>SYNERGY duct</t>
+        </is>
+      </c>
+      <c r="G516" t="inlineStr">
+        <is>
+          <t>THAICON TL-PD100-FR</t>
+        </is>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>pac_inv</t>
+        </is>
+      </c>
+      <c r="I516" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J516" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K516" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L516" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M516" t="n">
+        <v>36</v>
+      </c>
+      <c r="N516" t="inlineStr">
+        <is>
+          <t>10.55</t>
+        </is>
+      </c>
+      <c r="O516" t="n">
+        <v>100</v>
+      </c>
+      <c r="P516" t="n">
+        <v>137300</v>
+      </c>
+      <c r="Q516" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R516" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S516" t="inlineStr">
+        <is>
+          <t>SYNERGY duct Инвертор 36 BTU · до 100 м²</t>
+        </is>
+      </c>
+      <c r="T516" t="inlineStr">
+        <is>
+          <t>DC Inverter · Канальный · до 200 Па · проводной пульт · обогрев -15°С · R32 · 3 года</t>
+        </is>
+      </c>
+      <c r="U516" t="inlineStr">
+        <is>
+          <t>DC Inverter / R32|Канальный тип|Обогрев до -15°С|Охлаждение до -15°С|Встроенная дренажная помпа|Статическое давление до 200 Па|Проводной пульт в комплекте|Приёмник ИК-сигнала|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V516" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W516" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X516" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-synergy-duct.webp</t>
+        </is>
+      </c>
+      <c r="Y516" t="n">
+        <v>339</v>
+      </c>
     </row>
     <row r="517">
-      <c r="X517" s="1" t="n"/>
+      <c r="A517" t="n">
+        <v>1</v>
+      </c>
+      <c r="B517" t="n">
+        <v>1516</v>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>thaicon-pd140</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>SYNERGY duct</t>
+        </is>
+      </c>
+      <c r="G517" t="inlineStr">
+        <is>
+          <t>THAICON TL-PD140-FR4</t>
+        </is>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>pac_inv</t>
+        </is>
+      </c>
+      <c r="I517" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J517" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K517" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L517" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M517" t="n">
+        <v>48</v>
+      </c>
+      <c r="N517" t="inlineStr">
+        <is>
+          <t>14.07</t>
+        </is>
+      </c>
+      <c r="O517" t="n">
+        <v>130</v>
+      </c>
+      <c r="P517" t="n">
+        <v>171800</v>
+      </c>
+      <c r="Q517" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R517" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S517" t="inlineStr">
+        <is>
+          <t>SYNERGY duct Инвертор 48 BTU · до 130 м²</t>
+        </is>
+      </c>
+      <c r="T517" t="inlineStr">
+        <is>
+          <t>DC Inverter · Канальный · до 200 Па · проводной пульт · обогрев -15°С · R32 · 3 года</t>
+        </is>
+      </c>
+      <c r="U517" t="inlineStr">
+        <is>
+          <t>DC Inverter / R32|Канальный тип|Обогрев до -15°С|Охлаждение до -15°С|Встроенная дренажная помпа|Статическое давление до 200 Па|Проводной пульт в комплекте|Приёмник ИК-сигнала|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V517" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W517" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X517" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-synergy-duct.webp</t>
+        </is>
+      </c>
+      <c r="Y517" t="n">
+        <v>340</v>
+      </c>
     </row>
     <row r="518">
-      <c r="X518" s="1" t="n"/>
+      <c r="A518" t="n">
+        <v>1</v>
+      </c>
+      <c r="B518" t="n">
+        <v>1517</v>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>thaicon-pd170</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>SYNERGY duct</t>
+        </is>
+      </c>
+      <c r="G518" t="inlineStr">
+        <is>
+          <t>THAICON TL-PD170-FR4</t>
+        </is>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>pac_inv</t>
+        </is>
+      </c>
+      <c r="I518" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J518" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K518" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L518" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M518" t="n">
+        <v>60</v>
+      </c>
+      <c r="N518" t="inlineStr">
+        <is>
+          <t>16.12</t>
+        </is>
+      </c>
+      <c r="O518" t="n">
+        <v>160</v>
+      </c>
+      <c r="P518" t="n">
+        <v>186600</v>
+      </c>
+      <c r="Q518" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R518" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S518" t="inlineStr">
+        <is>
+          <t>SYNERGY duct Инвертор 60 BTU · до 160 м²</t>
+        </is>
+      </c>
+      <c r="T518" t="inlineStr">
+        <is>
+          <t>DC Inverter · Канальный · до 200 Па · проводной пульт · обогрев -15°С · R32 · 3 года</t>
+        </is>
+      </c>
+      <c r="U518" t="inlineStr">
+        <is>
+          <t>DC Inverter / R32|Канальный тип|Обогрев до -15°С|Охлаждение до -15°С|Встроенная дренажная помпа|Статическое давление до 200 Па|Проводной пульт в комплекте|Приёмник ИК-сигнала|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V518" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W518" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X518" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-synergy-duct.webp</t>
+        </is>
+      </c>
+      <c r="Y518" t="n">
+        <v>341</v>
+      </c>
     </row>
     <row r="519">
-      <c r="X519" s="1" t="n"/>
+      <c r="A519" t="n">
+        <v>1</v>
+      </c>
+      <c r="B519" t="n">
+        <v>1518</v>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>thaicon-pu50</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>SYNERGY floor-ceiling</t>
+        </is>
+      </c>
+      <c r="G519" t="inlineStr">
+        <is>
+          <t>THAICON TL-PU50-FR</t>
+        </is>
+      </c>
+      <c r="H519" t="inlineStr">
+        <is>
+          <t>pac_inv</t>
+        </is>
+      </c>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J519" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K519" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L519" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M519" t="n">
+        <v>18</v>
+      </c>
+      <c r="N519" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="O519" t="n">
+        <v>50</v>
+      </c>
+      <c r="P519" t="n">
+        <v>76900</v>
+      </c>
+      <c r="Q519" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R519" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S519" t="inlineStr">
+        <is>
+          <t>SYNERGY floor-ceiling Инвертор 18 BTU · до 50 м²</t>
+        </is>
+      </c>
+      <c r="T519" t="inlineStr">
+        <is>
+          <t>DC Inverter · Напольно-потолочный · 2 варианта монтажа · ИК-пульт · R32 · 3 года</t>
+        </is>
+      </c>
+      <c r="U519" t="inlineStr">
+        <is>
+          <t>DC Inverter / R32|Напольно-потолочный тип|Два варианта монтажа|Обогрев до -15°С|Охлаждение до -15°С|LED-дисплей|ИК-пульт в комплекте|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V519" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W519" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X519" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-synergy-floor-ceiling.webp</t>
+        </is>
+      </c>
+      <c r="Y519" t="n">
+        <v>342</v>
+      </c>
     </row>
     <row r="520">
-      <c r="X520" s="1" t="n"/>
+      <c r="A520" t="n">
+        <v>1</v>
+      </c>
+      <c r="B520" t="n">
+        <v>1519</v>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>thaicon-pu70</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>SYNERGY floor-ceiling</t>
+        </is>
+      </c>
+      <c r="G520" t="inlineStr">
+        <is>
+          <t>THAICON TL-PU70-FR</t>
+        </is>
+      </c>
+      <c r="H520" t="inlineStr">
+        <is>
+          <t>pac_inv</t>
+        </is>
+      </c>
+      <c r="I520" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J520" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K520" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L520" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M520" t="n">
+        <v>24</v>
+      </c>
+      <c r="N520" t="inlineStr">
+        <is>
+          <t>7.03</t>
+        </is>
+      </c>
+      <c r="O520" t="n">
+        <v>65</v>
+      </c>
+      <c r="P520" t="n">
+        <v>95100</v>
+      </c>
+      <c r="Q520" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R520" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S520" t="inlineStr">
+        <is>
+          <t>SYNERGY floor-ceiling Инвертор 24 BTU · до 65 м²</t>
+        </is>
+      </c>
+      <c r="T520" t="inlineStr">
+        <is>
+          <t>DC Inverter · Напольно-потолочный · 2 варианта монтажа · ИК-пульт · R32 · 3 года</t>
+        </is>
+      </c>
+      <c r="U520" t="inlineStr">
+        <is>
+          <t>DC Inverter / R32|Напольно-потолочный тип|Два варианта монтажа|Обогрев до -15°С|Охлаждение до -15°С|LED-дисплей|ИК-пульт в комплекте|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V520" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W520" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X520" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-synergy-floor-ceiling.webp</t>
+        </is>
+      </c>
+      <c r="Y520" t="n">
+        <v>343</v>
+      </c>
     </row>
     <row r="521">
-      <c r="X521" s="1" t="n"/>
+      <c r="A521" t="n">
+        <v>1</v>
+      </c>
+      <c r="B521" t="n">
+        <v>1520</v>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>thaicon-pu100</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>SYNERGY floor-ceiling</t>
+        </is>
+      </c>
+      <c r="G521" t="inlineStr">
+        <is>
+          <t>THAICON TL-PU100-FR</t>
+        </is>
+      </c>
+      <c r="H521" t="inlineStr">
+        <is>
+          <t>pac_inv</t>
+        </is>
+      </c>
+      <c r="I521" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J521" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K521" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L521" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M521" t="n">
+        <v>36</v>
+      </c>
+      <c r="N521" t="inlineStr">
+        <is>
+          <t>10.55</t>
+        </is>
+      </c>
+      <c r="O521" t="n">
+        <v>100</v>
+      </c>
+      <c r="P521" t="n">
+        <v>129700</v>
+      </c>
+      <c r="Q521" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R521" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S521" t="inlineStr">
+        <is>
+          <t>SYNERGY floor-ceiling Инвертор 36 BTU · до 100 м²</t>
+        </is>
+      </c>
+      <c r="T521" t="inlineStr">
+        <is>
+          <t>DC Inverter · Напольно-потолочный · 2 варианта монтажа · ИК-пульт · R32 · 3 года</t>
+        </is>
+      </c>
+      <c r="U521" t="inlineStr">
+        <is>
+          <t>DC Inverter / R32|Напольно-потолочный тип|Два варианта монтажа|Обогрев до -15°С|Охлаждение до -15°С|LED-дисплей|ИК-пульт в комплекте|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V521" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W521" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X521" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-synergy-floor-ceiling.webp</t>
+        </is>
+      </c>
+      <c r="Y521" t="n">
+        <v>344</v>
+      </c>
     </row>
     <row r="522">
-      <c r="X522" s="1" t="n"/>
+      <c r="A522" t="n">
+        <v>1</v>
+      </c>
+      <c r="B522" t="n">
+        <v>1521</v>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>thaicon-pu140</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>SYNERGY floor-ceiling</t>
+        </is>
+      </c>
+      <c r="G522" t="inlineStr">
+        <is>
+          <t>THAICON TL-PU140-FR4</t>
+        </is>
+      </c>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>pac_inv</t>
+        </is>
+      </c>
+      <c r="I522" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J522" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K522" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L522" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M522" t="n">
+        <v>48</v>
+      </c>
+      <c r="N522" t="inlineStr">
+        <is>
+          <t>14.07</t>
+        </is>
+      </c>
+      <c r="O522" t="n">
+        <v>130</v>
+      </c>
+      <c r="P522" t="n">
+        <v>166300</v>
+      </c>
+      <c r="Q522" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R522" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S522" t="inlineStr">
+        <is>
+          <t>SYNERGY floor-ceiling Инвертор 48 BTU · до 130 м²</t>
+        </is>
+      </c>
+      <c r="T522" t="inlineStr">
+        <is>
+          <t>DC Inverter · Напольно-потолочный · 2 варианта монтажа · ИК-пульт · R32 · 3 года</t>
+        </is>
+      </c>
+      <c r="U522" t="inlineStr">
+        <is>
+          <t>DC Inverter / R32|Напольно-потолочный тип|Два варианта монтажа|Обогрев до -15°С|Охлаждение до -15°С|LED-дисплей|ИК-пульт в комплекте|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V522" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W522" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X522" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-synergy-floor-ceiling.webp</t>
+        </is>
+      </c>
+      <c r="Y522" t="n">
+        <v>345</v>
+      </c>
     </row>
     <row r="523">
-      <c r="X523" s="1" t="n"/>
+      <c r="A523" t="n">
+        <v>1</v>
+      </c>
+      <c r="B523" t="n">
+        <v>1522</v>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>thaicon-pu170</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>thai</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>THAICON</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>SYNERGY floor-ceiling</t>
+        </is>
+      </c>
+      <c r="G523" t="inlineStr">
+        <is>
+          <t>THAICON TL-PU170-FR4</t>
+        </is>
+      </c>
+      <c r="H523" t="inlineStr">
+        <is>
+          <t>pac_inv</t>
+        </is>
+      </c>
+      <c r="I523" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="J523" t="inlineStr">
+        <is>
+          <t>TCL</t>
+        </is>
+      </c>
+      <c r="K523" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="L523" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M523" t="n">
+        <v>60</v>
+      </c>
+      <c r="N523" t="inlineStr">
+        <is>
+          <t>16.12</t>
+        </is>
+      </c>
+      <c r="O523" t="n">
+        <v>160</v>
+      </c>
+      <c r="P523" t="n">
+        <v>183200</v>
+      </c>
+      <c r="Q523" t="inlineStr">
+        <is>
+          <t>in_stock</t>
+        </is>
+      </c>
+      <c r="R523" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="S523" t="inlineStr">
+        <is>
+          <t>SYNERGY floor-ceiling Инвертор 60 BTU · до 160 м²</t>
+        </is>
+      </c>
+      <c r="T523" t="inlineStr">
+        <is>
+          <t>DC Inverter · Напольно-потолочный · 2 варианта монтажа · ИК-пульт · R32 · 3 года</t>
+        </is>
+      </c>
+      <c r="U523" t="inlineStr">
+        <is>
+          <t>DC Inverter / R32|Напольно-потолочный тип|Два варианта монтажа|Обогрев до -15°С|Охлаждение до -15°С|LED-дисплей|ИК-пульт в комплекте|Гарантия - 3 года</t>
+        </is>
+      </c>
+      <c r="V523" t="inlineStr">
+        <is>
+          <t>GMCC</t>
+        </is>
+      </c>
+      <c r="W523" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="X523" s="1" t="inlineStr">
+        <is>
+          <t>thaicon-synergy-floor-ceiling.webp</t>
+        </is>
+      </c>
+      <c r="Y523" t="n">
+        <v>346</v>
+      </c>
     </row>
     <row r="524">
       <c r="X524" s="1" t="n"/>
@@ -70191,114 +73664,6 @@
     </row>
     <row r="4877">
       <c r="X4877" s="1" t="n"/>
-    </row>
-    <row r="4878">
-      <c r="X4878" s="1" t="n"/>
-    </row>
-    <row r="4879">
-      <c r="X4879" s="1" t="n"/>
-    </row>
-    <row r="4880">
-      <c r="X4880" s="1" t="n"/>
-    </row>
-    <row r="4881">
-      <c r="X4881" s="1" t="n"/>
-    </row>
-    <row r="4882">
-      <c r="X4882" s="1" t="n"/>
-    </row>
-    <row r="4883">
-      <c r="X4883" s="1" t="n"/>
-    </row>
-    <row r="4884">
-      <c r="X4884" s="1" t="n"/>
-    </row>
-    <row r="4885">
-      <c r="X4885" s="1" t="n"/>
-    </row>
-    <row r="4886">
-      <c r="X4886" s="1" t="n"/>
-    </row>
-    <row r="4887">
-      <c r="X4887" s="1" t="n"/>
-    </row>
-    <row r="4888">
-      <c r="X4888" s="1" t="n"/>
-    </row>
-    <row r="4889">
-      <c r="X4889" s="1" t="n"/>
-    </row>
-    <row r="4890">
-      <c r="X4890" s="1" t="n"/>
-    </row>
-    <row r="4891">
-      <c r="X4891" s="1" t="n"/>
-    </row>
-    <row r="4892">
-      <c r="X4892" s="1" t="n"/>
-    </row>
-    <row r="4893">
-      <c r="X4893" s="1" t="n"/>
-    </row>
-    <row r="4894">
-      <c r="X4894" s="1" t="n"/>
-    </row>
-    <row r="4895">
-      <c r="X4895" s="1" t="n"/>
-    </row>
-    <row r="4896">
-      <c r="X4896" s="1" t="n"/>
-    </row>
-    <row r="4897">
-      <c r="X4897" s="1" t="n"/>
-    </row>
-    <row r="4898">
-      <c r="X4898" s="1" t="n"/>
-    </row>
-    <row r="4899">
-      <c r="X4899" s="1" t="n"/>
-    </row>
-    <row r="4900">
-      <c r="X4900" s="1" t="n"/>
-    </row>
-    <row r="4901">
-      <c r="X4901" s="1" t="n"/>
-    </row>
-    <row r="4902">
-      <c r="X4902" s="1" t="n"/>
-    </row>
-    <row r="4903">
-      <c r="X4903" s="1" t="n"/>
-    </row>
-    <row r="4904">
-      <c r="X4904" s="1" t="n"/>
-    </row>
-    <row r="4905">
-      <c r="X4905" s="1" t="n"/>
-    </row>
-    <row r="4906">
-      <c r="X4906" s="1" t="n"/>
-    </row>
-    <row r="4907">
-      <c r="X4907" s="1" t="n"/>
-    </row>
-    <row r="4908">
-      <c r="X4908" s="1" t="n"/>
-    </row>
-    <row r="4909">
-      <c r="X4909" s="1" t="n"/>
-    </row>
-    <row r="4910">
-      <c r="X4910" s="1" t="n"/>
-    </row>
-    <row r="4911">
-      <c r="X4911" s="1" t="n"/>
-    </row>
-    <row r="4912">
-      <c r="X4912" s="1" t="n"/>
-    </row>
-    <row r="4913">
-      <c r="X4913" s="1" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y4913"/>

</xml_diff>